<commit_message>
include factual audit links in calendar Council exports
</commit_message>
<xml_diff>
--- a/docs/ui-calendar-eight/KyCalendar-Council.xlsx
+++ b/docs/ui-calendar-eight/KyCalendar-Council.xlsx
@@ -69922,6 +69922,30 @@
     <row r="14">
       <c t="inlineStr">
         <is>
+          <t xml:space="preserve">Factual audit, round 1</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">{"file": "round1-disagreement-audit.json", "sha256": "9726720ae73366045975f8f89a089f453a1e3804167446f6e1da703379216f34"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Factual audit, round 2</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">{"file": "round2-disagreement-audit.json", "sha256": "736e06043a23d8da39a3fbb2fe1aef478171f43b41bd09d348e8874cd415948d"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c t="inlineStr">
+        <is>
           <t xml:space="preserve">Review limitation, round 3</t>
         </is>
       </c>
@@ -69931,7 +69955,7 @@
         </is>
       </c>
     </row>
-    <row r="15">
+    <row r="17">
       <c t="inlineStr">
         <is>
           <t xml:space="preserve">Review limitation, round 3</t>
@@ -69943,7 +69967,7 @@
         </is>
       </c>
     </row>
-    <row r="16">
+    <row r="18">
       <c t="inlineStr">
         <is>
           <t xml:space="preserve">Review limitation, round 3</t>
@@ -69952,6 +69976,18 @@
       <c t="inlineStr">
         <is>
           <t xml:space="preserve">Raw scores and all vectors unchanged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Factual audit, round 3</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">{"file": "round3-disagreement-audit.json", "sha256": "6664b0209f40e1b189b143a0a76dc8b5c42680a722dd044e126f6cf11ea56c5f"}</t>
         </is>
       </c>
     </row>

</xml_diff>